<commit_message>
Updated EST model - 2025-11-05 19:10
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C8B0A46-9C39-4C32-80BB-622F5F66D4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3FC00B5A-827F-4363-94E6-F3171C09E532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5715,7 +5715,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02121A9A-9509-4439-8806-CD6AA93B92D3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C00310DD-1CB4-486C-A552-DBB361784DD7}">
   <dimension ref="B9:M20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6118,7 +6118,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BD906F5-DE0F-4F85-B69A-66E82B7A4DD5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CE11FA-424D-4175-8D51-C3D4BFFCF9D6}">
   <dimension ref="B9:Z20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6890,7 +6890,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23C4B6D3-E927-481D-8E70-B0D3EEEF9328}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFAEA120-4665-4DDA-A182-AF6A462EBBA9}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>